<commit_message>
Big update cập nhật Adroind app
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/PaymentStatus_template.xlsx
+++ b/MPR_Managerment/Templates/PaymentStatus_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c02630c4a1efac79/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Git\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{E55CEA31-F453-4A94-9B01-A37129F803CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0026509E-049B-49DE-A607-38A8D02392C5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0EAC5D-91DC-43BD-9118-883AC51B4CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{30FEABF5-A9B5-4797-85DA-5F695B535E1F}"/>
   </bookViews>
@@ -1579,7 +1579,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1609,6 +1609,14 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1693,9 +1701,6 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1708,19 +1713,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1729,23 +1722,38 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2361,311 +2369,311 @@
   <dimension ref="A1:U9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.75" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="16.875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18.75" style="3" customWidth="1"/>
-    <col min="6" max="6" width="19.125" style="2" customWidth="1"/>
-    <col min="7" max="19" width="31.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="30.125" style="2" customWidth="1"/>
-    <col min="21" max="21" width="24.75" style="2" customWidth="1"/>
-    <col min="22" max="23" width="9.75" style="2" customWidth="1"/>
-    <col min="24" max="24" width="12" style="2" customWidth="1"/>
-    <col min="25" max="16384" width="9" style="2"/>
+    <col min="1" max="1" width="5.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.75" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.75" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.125" style="1" customWidth="1"/>
+    <col min="7" max="19" width="31.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="30.125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="24.75" style="1" customWidth="1"/>
+    <col min="22" max="23" width="9.75" style="1" customWidth="1"/>
+    <col min="24" max="24" width="12" style="1" customWidth="1"/>
+    <col min="25" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="23.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+      <c r="U1" s="9"/>
     </row>
     <row r="3" spans="1:21">
-      <c r="U3" s="4" t="s">
+      <c r="U3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="16.5" customHeight="1">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="8">
         <v>2025</v>
       </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5" t="s">
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="T4" s="5" t="s">
+      <c r="T4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="U4" s="5" t="s">
+      <c r="U4" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="9">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="5">
         <v>46023</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="5">
         <v>46054</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="5">
         <v>46082</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="5">
         <v>46113</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="5">
         <v>46143</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="5">
         <v>46174</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="5">
         <v>46204</v>
       </c>
-      <c r="N5" s="9">
+      <c r="N5" s="5">
         <v>46235</v>
       </c>
-      <c r="O5" s="9">
+      <c r="O5" s="5">
         <v>46266</v>
       </c>
-      <c r="P5" s="9">
+      <c r="P5" s="5">
         <v>46296</v>
       </c>
-      <c r="Q5" s="9">
+      <c r="Q5" s="5">
         <v>46327</v>
       </c>
-      <c r="R5" s="9">
+      <c r="R5" s="5">
         <v>46357</v>
       </c>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
     </row>
     <row r="6" spans="1:21" ht="57" customHeight="1">
-      <c r="A6" s="10">
+      <c r="A6" s="4">
         <v>1</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="L6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="M6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="P6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="Q6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="11" t="s">
+      <c r="R6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="S6" s="12" t="s">
+      <c r="S6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T6" s="12" t="s">
+      <c r="T6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="U6" s="10"/>
+      <c r="U6" s="4"/>
     </row>
     <row r="7" spans="1:21" ht="14.25" hidden="1" customHeight="1">
-      <c r="A7" s="10"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="10" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
-      <c r="R7" s="12"/>
-      <c r="S7" s="12"/>
-      <c r="T7" s="12"/>
-      <c r="U7" s="10"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="4"/>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="10">
+      <c r="A8" s="4">
         <v>2</v>
       </c>
-      <c r="B8" s="15"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="18"/>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="12"/>
-      <c r="S8" s="12"/>
-      <c r="T8" s="12"/>
-      <c r="U8" s="10"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="4"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="12" t="s">
+      <c r="D9" s="4"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="J9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="K9" s="12" t="s">
+      <c r="K9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="L9" s="12" t="s">
+      <c r="L9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="M9" s="12" t="s">
+      <c r="M9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="O9" s="12" t="s">
+      <c r="O9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="P9" s="12" t="s">
+      <c r="P9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="Q9" s="12" t="s">
+      <c r="Q9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="R9" s="12" t="s">
+      <c r="R9" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="S9" s="12" t="s">
+      <c r="S9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T9" s="12" t="s">
+      <c r="T9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="U9" s="12">
+      <c r="U9" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>